<commit_message>
test(ppe): ejemplo del mayor con las columnas nuevas (detalle, referencia, clasificación)
El dataset del mayor ahora tiene los campos «Descripción del movimiento», «Referencia»
y «Clasificación del movimiento»; el archivo de ejemplo RQ-010_mayor.xlsx se regenera con
esos rótulos para que test_aud_ejemplos_lote1 auto-mapee todos los campos.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G6VP4biUU9DJHYQEXimtNg
</commit_message>
<xml_diff>
--- a/frontend/public/ejemplos/ppe_propiedad_planta/RQ-010_mayor.xlsx
+++ b/frontend/public/ejemplos/ppe_propiedad_planta/RQ-010_mayor.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Datos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -492,18 +492,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -519,37 +522,52 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
+          <t>Descripción del movimiento</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Referencia</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
           <t>Fecha del movimiento</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>N° de comprobante</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>N° de documento</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Tipo de asiento</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Debe</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Haber</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Importe (valor neto del movimiento)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Clasificación del movimiento (Adición/Ajuste/Venta/Depreciación)</t>
         </is>
       </c>
     </row>
@@ -564,41 +582,44 @@
           <t>Muebles y enseres</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>01/04/2025</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>CMP-120</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>FAC-5521</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>VO</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>12000</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>12000</t>
         </is>
       </c>
+      <c r="L2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -611,41 +632,44 @@
           <t>Vehículos</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>30/06/2025</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr"/>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>CMP-215</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>ND-048</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>VO</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>30000</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>-30000</t>
         </is>
       </c>
+      <c r="L3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -658,41 +682,44 @@
           <t>Depreciación acumulada</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>31/12/2025</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>CMP-312</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>AJ-900</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>ADJ</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>28000</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>-28000</t>
         </is>
       </c>
+      <c r="L4" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -705,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -794,7 +821,7 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Fecha del movimiento</t>
+          <t>Descripción del movimiento</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -807,7 +834,7 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>N° de comprobante</t>
+          <t>Referencia</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -820,7 +847,7 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>N° de documento</t>
+          <t>Fecha del movimiento</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -833,7 +860,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Tipo de asiento</t>
+          <t>N° de comprobante</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -846,7 +873,7 @@
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>Debe</t>
+          <t>N° de documento</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -859,7 +886,7 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Haber</t>
+          <t>Tipo de asiento</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
@@ -872,15 +899,54 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
+          <t>Debe</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Haber</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
           <t>Importe (valor neto del movimiento)</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>Opcional</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr"/>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Clasificación del movimiento (Adición/Ajuste/Venta/Depreciación)</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>